<commit_message>
Put all normal ad budget on FULLMARKS until other stores launch
Other stores' share (STORE_R) is 0 until the user confirms they will run
ads, so Oct-Apr normal operations go entirely to FULLMARKS (October
1,052,086 yen). Event reserves stay separate. October brand ratios updated
to September results.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EFkMa7pBd48FUqtUrcDcW8
</commit_message>
<xml_diff>
--- a/reports/広告予算計画_2026-09改訂.xlsx
+++ b/reports/広告予算計画_2026-09改訂.xlsx
@@ -575,11 +575,11 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>HOUDINI STORE 9月末開店 / NORRONA・PU 10月開店 → 10月から各15%、FULLMARKS 55%</t>
+          <t>他ECは実施が決まるまで0%（2026-09-28 ユーザー指示）。通常運用は全額 FULLMARKS。開店が決まったら各15%などに変更</t>
         </is>
       </c>
     </row>
@@ -1010,11 +1010,11 @@
         <v>0.27</v>
       </c>
       <c r="C40" s="5" t="n">
-        <v>0.2</v>
+        <v>0.26</v>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>売上の7割。Google指名 ROAS 12〜13、Meta RTG 5.0（9月第1週）。HOUDINI STORE稼働後は縮小</t>
+          <t>広告売上の半分以上（9月 ROAS 11.8）。FULLMARKS で継続</t>
         </is>
       </c>
     </row>
@@ -1028,11 +1028,11 @@
         <v>0.3</v>
       </c>
       <c r="C41" s="5" t="n">
-        <v>0.28</v>
+        <v>0.23</v>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>通常価格品のみ（アウトレットは広告しない）。PLA 4,000円/日＋Metaカタログ9本 5,000円/日</t>
+          <t>通常価格品のみ（アウトレットは広告しない）。9月 ROAS: カタログ 4.6 / ショッピング 2.5。ショッピングを絞る</t>
         </is>
       </c>
     </row>
@@ -1050,7 +1050,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>ROAS 9〜10の安定枠</t>
+          <t>9月 ROAS 16.2 の安定枠</t>
         </is>
       </c>
     </row>
@@ -1064,11 +1064,11 @@
         <v>0.09</v>
       </c>
       <c r="C43" s="5" t="n">
-        <v>0.12</v>
+        <v>0.11</v>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>9月売上構成比13%に上昇。専用ストア無し</t>
+          <t>9月 ROAS 3.8。10月以降やや厚く</t>
         </is>
       </c>
     </row>
@@ -1082,11 +1082,11 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="C44" s="5" t="n">
-        <v>0.06</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>ROAS 2前後。NORRONA STORE移管で最小化</t>
+          <t>9月 ROAS 4.1（8月 1.0 から改善）。FULLMARKS で継続</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
         <v>0.05</v>
       </c>
       <c r="C45" s="5" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
@@ -1216,7 +1216,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>通常運用＝上限−実績−9月−イベント予備費 を10〜4月の比率で配分。10月から HOUDINI / NORRONA / PU STORE が各15%。</t>
+          <t>通常運用＝上限−実績−9月−イベント予備費 を10〜4月の比率で配分。他ECは実施が決まるまで0（前提!B5）で、全額 FULLMARKS。</t>
         </is>
       </c>
     </row>
@@ -1603,7 +1603,7 @@
       </c>
       <c r="M10" s="17" t="inlineStr">
         <is>
-          <t>3ストア稼働・広告開始。勝負月</t>
+          <t>勝負月</t>
         </is>
       </c>
     </row>
@@ -2124,7 +2124,7 @@
       </c>
       <c r="K5" s="17" t="inlineStr">
         <is>
-          <t>売上の7割。Google指名 ROAS 12〜13、Meta RTG 5.0（9月第1週）。HOUDINI STORE稼働後は縮小</t>
+          <t>広告売上の半分以上（9月 ROAS 11.8）。FULLMARKS で継続</t>
         </is>
       </c>
     </row>
@@ -2172,7 +2172,7 @@
       </c>
       <c r="K6" s="17" t="inlineStr">
         <is>
-          <t>通常価格品のみ（アウトレットは広告しない）。PLA 4,000円/日＋Metaカタログ9本 5,000円/日</t>
+          <t>通常価格品のみ（アウトレットは広告しない）。9月 ROAS: カタログ 4.6 / ショッピング 2.5。ショッピングを絞る</t>
         </is>
       </c>
     </row>
@@ -2220,7 +2220,7 @@
       </c>
       <c r="K7" s="17" t="inlineStr">
         <is>
-          <t>ROAS 9〜10の安定枠</t>
+          <t>9月 ROAS 16.2 の安定枠</t>
         </is>
       </c>
     </row>
@@ -2268,7 +2268,7 @@
       </c>
       <c r="K8" s="17" t="inlineStr">
         <is>
-          <t>9月売上構成比13%に上昇。専用ストア無し</t>
+          <t>9月 ROAS 3.8。10月以降やや厚く</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="K9" s="17" t="inlineStr">
         <is>
-          <t>ROAS 2前後。NORRONA STORE移管で最小化</t>
+          <t>9月 ROAS 4.1（8月 1.0 から改善）。FULLMARKS で継続</t>
         </is>
       </c>
     </row>
@@ -2608,7 +2608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T28"/>
+  <dimension ref="A1:T19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -2643,7 +2643,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>緑＝新設キャンペーン。3ストアは10月から 指名45% / ショッピング30% / カタログ・RTG25% の標準構成。ショッピング・カタログはすべて通常価格品のみ（アウトレット除外）。イベント予備費は欄外。</t>
+          <t>緑＝新設キャンペーン。他ECは実施が決まるまで載せない（前提!B5 を0より大きくすると 指名45% / ショッピング30% / カタログ・RTG25% で行が出る）。ショッピング・カタログはすべて通常価格品のみ（アウトレット除外）。イベント予備費は欄外。</t>
         </is>
       </c>
     </row>
@@ -3954,899 +3954,125 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="29" t="inlineStr">
-        <is>
-          <t>HOUDINI STORE</t>
-        </is>
-      </c>
-      <c r="B18" s="29" t="inlineStr">
-        <is>
-          <t>ストア全体</t>
-        </is>
-      </c>
-      <c r="C18" s="29" t="inlineStr">
-        <is>
-          <t>Google</t>
-        </is>
-      </c>
-      <c r="D18" s="29" t="inlineStr">
-        <is>
-          <t>【新設】指名検索</t>
-        </is>
-      </c>
-      <c r="E18" s="30">
-        <f>ROUND(M18/30,-2)</f>
-        <v/>
-      </c>
-      <c r="F18" s="30">
-        <f>ROUND(N18/31,-2)</f>
-        <v/>
-      </c>
-      <c r="G18" s="30">
-        <f>ROUND(O18/30,-2)</f>
-        <v/>
-      </c>
-      <c r="H18" s="30">
-        <f>ROUND(P18/31,-2)</f>
-        <v/>
-      </c>
-      <c r="I18" s="30">
-        <f>ROUND(Q18/31,-2)</f>
-        <v/>
-      </c>
-      <c r="J18" s="30">
-        <f>ROUND(R18/28,-2)</f>
-        <v/>
-      </c>
-      <c r="K18" s="30">
-        <f>ROUND(S18/31,-2)</f>
-        <v/>
-      </c>
-      <c r="L18" s="30">
-        <f>ROUND(T18/30,-2)</f>
-        <v/>
-      </c>
-      <c r="M18" s="30">
-        <f>ROUND(月別予算!$D$9*0.45,0)</f>
-        <v/>
-      </c>
-      <c r="N18" s="30">
-        <f>ROUND(月別予算!$D$10*0.45,0)</f>
-        <v/>
-      </c>
-      <c r="O18" s="30">
-        <f>ROUND(月別予算!$D$11*0.45,0)</f>
-        <v/>
-      </c>
-      <c r="P18" s="30">
-        <f>ROUND(月別予算!$D$12*0.45,0)</f>
-        <v/>
-      </c>
-      <c r="Q18" s="30">
-        <f>ROUND(月別予算!$D$13*0.45,0)</f>
-        <v/>
-      </c>
-      <c r="R18" s="30">
-        <f>ROUND(月別予算!$D$14*0.45,0)</f>
-        <v/>
-      </c>
-      <c r="S18" s="30">
-        <f>ROUND(月別予算!$D$15*0.45,0)</f>
-        <v/>
-      </c>
-      <c r="T18" s="30">
-        <f>ROUND(月別予算!$D$16*0.45,0)</f>
+      <c r="A18" s="21" t="inlineStr">
+        <is>
+          <t>合計（通常運用）</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="n"/>
+      <c r="C18" s="18" t="n"/>
+      <c r="D18" s="18" t="n"/>
+      <c r="E18" s="22">
+        <f>SUM(E4:E17)</f>
+        <v/>
+      </c>
+      <c r="F18" s="22">
+        <f>SUM(F4:F17)</f>
+        <v/>
+      </c>
+      <c r="G18" s="22">
+        <f>SUM(G4:G17)</f>
+        <v/>
+      </c>
+      <c r="H18" s="22">
+        <f>SUM(H4:H17)</f>
+        <v/>
+      </c>
+      <c r="I18" s="22">
+        <f>SUM(I4:I17)</f>
+        <v/>
+      </c>
+      <c r="J18" s="22">
+        <f>SUM(J4:J17)</f>
+        <v/>
+      </c>
+      <c r="K18" s="22">
+        <f>SUM(K4:K17)</f>
+        <v/>
+      </c>
+      <c r="L18" s="22">
+        <f>SUM(L4:L17)</f>
+        <v/>
+      </c>
+      <c r="M18" s="22">
+        <f>SUM(M4:M17)</f>
+        <v/>
+      </c>
+      <c r="N18" s="22">
+        <f>SUM(N4:N17)</f>
+        <v/>
+      </c>
+      <c r="O18" s="22">
+        <f>SUM(O4:O17)</f>
+        <v/>
+      </c>
+      <c r="P18" s="22">
+        <f>SUM(P4:P17)</f>
+        <v/>
+      </c>
+      <c r="Q18" s="22">
+        <f>SUM(Q4:Q17)</f>
+        <v/>
+      </c>
+      <c r="R18" s="22">
+        <f>SUM(R4:R17)</f>
+        <v/>
+      </c>
+      <c r="S18" s="22">
+        <f>SUM(S4:S17)</f>
+        <v/>
+      </c>
+      <c r="T18" s="22">
+        <f>SUM(T4:T17)</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="29" t="inlineStr">
-        <is>
-          <t>HOUDINI STORE</t>
-        </is>
-      </c>
-      <c r="B19" s="29" t="inlineStr">
-        <is>
-          <t>ストア全体</t>
-        </is>
-      </c>
-      <c r="C19" s="29" t="inlineStr">
-        <is>
-          <t>Google</t>
-        </is>
-      </c>
-      <c r="D19" s="29" t="inlineStr">
-        <is>
-          <t>【新設】ショッピング(通常価格のみ)</t>
-        </is>
-      </c>
-      <c r="E19" s="30">
-        <f>ROUND(M19/30,-2)</f>
-        <v/>
-      </c>
-      <c r="F19" s="30">
-        <f>ROUND(N19/31,-2)</f>
-        <v/>
-      </c>
-      <c r="G19" s="30">
-        <f>ROUND(O19/30,-2)</f>
-        <v/>
-      </c>
-      <c r="H19" s="30">
-        <f>ROUND(P19/31,-2)</f>
-        <v/>
-      </c>
-      <c r="I19" s="30">
-        <f>ROUND(Q19/31,-2)</f>
-        <v/>
-      </c>
-      <c r="J19" s="30">
-        <f>ROUND(R19/28,-2)</f>
-        <v/>
-      </c>
-      <c r="K19" s="30">
-        <f>ROUND(S19/31,-2)</f>
-        <v/>
-      </c>
-      <c r="L19" s="30">
-        <f>ROUND(T19/30,-2)</f>
-        <v/>
-      </c>
-      <c r="M19" s="30">
-        <f>ROUND(月別予算!$D$9*0.3,0)</f>
-        <v/>
-      </c>
-      <c r="N19" s="30">
-        <f>ROUND(月別予算!$D$10*0.3,0)</f>
-        <v/>
-      </c>
-      <c r="O19" s="30">
-        <f>ROUND(月別予算!$D$11*0.3,0)</f>
-        <v/>
-      </c>
-      <c r="P19" s="30">
-        <f>ROUND(月別予算!$D$12*0.3,0)</f>
-        <v/>
-      </c>
-      <c r="Q19" s="30">
-        <f>ROUND(月別予算!$D$13*0.3,0)</f>
-        <v/>
-      </c>
-      <c r="R19" s="30">
-        <f>ROUND(月別予算!$D$14*0.3,0)</f>
-        <v/>
-      </c>
-      <c r="S19" s="30">
-        <f>ROUND(月別予算!$D$15*0.3,0)</f>
-        <v/>
-      </c>
-      <c r="T19" s="30">
-        <f>ROUND(月別予算!$D$16*0.3,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="29" t="inlineStr">
-        <is>
-          <t>HOUDINI STORE</t>
-        </is>
-      </c>
-      <c r="B20" s="29" t="inlineStr">
-        <is>
-          <t>ストア全体</t>
-        </is>
-      </c>
-      <c r="C20" s="29" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
-      <c r="D20" s="29" t="inlineStr">
-        <is>
-          <t>【新設】カタログ/リターゲティング</t>
-        </is>
-      </c>
-      <c r="E20" s="30">
-        <f>ROUND(M20/30,-2)</f>
-        <v/>
-      </c>
-      <c r="F20" s="30">
-        <f>ROUND(N20/31,-2)</f>
-        <v/>
-      </c>
-      <c r="G20" s="30">
-        <f>ROUND(O20/30,-2)</f>
-        <v/>
-      </c>
-      <c r="H20" s="30">
-        <f>ROUND(P20/31,-2)</f>
-        <v/>
-      </c>
-      <c r="I20" s="30">
-        <f>ROUND(Q20/31,-2)</f>
-        <v/>
-      </c>
-      <c r="J20" s="30">
-        <f>ROUND(R20/28,-2)</f>
-        <v/>
-      </c>
-      <c r="K20" s="30">
-        <f>ROUND(S20/31,-2)</f>
-        <v/>
-      </c>
-      <c r="L20" s="30">
-        <f>ROUND(T20/30,-2)</f>
-        <v/>
-      </c>
-      <c r="M20" s="30">
-        <f>ROUND(月別予算!$D$9*0.25,0)</f>
-        <v/>
-      </c>
-      <c r="N20" s="30">
-        <f>ROUND(月別予算!$D$10*0.25,0)</f>
-        <v/>
-      </c>
-      <c r="O20" s="30">
-        <f>ROUND(月別予算!$D$11*0.25,0)</f>
-        <v/>
-      </c>
-      <c r="P20" s="30">
-        <f>ROUND(月別予算!$D$12*0.25,0)</f>
-        <v/>
-      </c>
-      <c r="Q20" s="30">
-        <f>ROUND(月別予算!$D$13*0.25,0)</f>
-        <v/>
-      </c>
-      <c r="R20" s="30">
-        <f>ROUND(月別予算!$D$14*0.25,0)</f>
-        <v/>
-      </c>
-      <c r="S20" s="30">
-        <f>ROUND(月別予算!$D$15*0.25,0)</f>
-        <v/>
-      </c>
-      <c r="T20" s="30">
-        <f>ROUND(月別予算!$D$16*0.25,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="29" t="inlineStr">
-        <is>
-          <t>NORRONA STORE</t>
-        </is>
-      </c>
-      <c r="B21" s="29" t="inlineStr">
-        <is>
-          <t>ストア全体</t>
-        </is>
-      </c>
-      <c r="C21" s="29" t="inlineStr">
-        <is>
-          <t>Google</t>
-        </is>
-      </c>
-      <c r="D21" s="29" t="inlineStr">
-        <is>
-          <t>【新設】指名検索</t>
-        </is>
-      </c>
-      <c r="E21" s="30">
-        <f>ROUND(M21/30,-2)</f>
-        <v/>
-      </c>
-      <c r="F21" s="30">
-        <f>ROUND(N21/31,-2)</f>
-        <v/>
-      </c>
-      <c r="G21" s="30">
-        <f>ROUND(O21/30,-2)</f>
-        <v/>
-      </c>
-      <c r="H21" s="30">
-        <f>ROUND(P21/31,-2)</f>
-        <v/>
-      </c>
-      <c r="I21" s="30">
-        <f>ROUND(Q21/31,-2)</f>
-        <v/>
-      </c>
-      <c r="J21" s="30">
-        <f>ROUND(R21/28,-2)</f>
-        <v/>
-      </c>
-      <c r="K21" s="30">
-        <f>ROUND(S21/31,-2)</f>
-        <v/>
-      </c>
-      <c r="L21" s="30">
-        <f>ROUND(T21/30,-2)</f>
-        <v/>
-      </c>
-      <c r="M21" s="30">
-        <f>ROUND(月別予算!$E$9*0.45,0)</f>
-        <v/>
-      </c>
-      <c r="N21" s="30">
-        <f>ROUND(月別予算!$E$10*0.45,0)</f>
-        <v/>
-      </c>
-      <c r="O21" s="30">
-        <f>ROUND(月別予算!$E$11*0.45,0)</f>
-        <v/>
-      </c>
-      <c r="P21" s="30">
-        <f>ROUND(月別予算!$E$12*0.45,0)</f>
-        <v/>
-      </c>
-      <c r="Q21" s="30">
-        <f>ROUND(月別予算!$E$13*0.45,0)</f>
-        <v/>
-      </c>
-      <c r="R21" s="30">
-        <f>ROUND(月別予算!$E$14*0.45,0)</f>
-        <v/>
-      </c>
-      <c r="S21" s="30">
-        <f>ROUND(月別予算!$E$15*0.45,0)</f>
-        <v/>
-      </c>
-      <c r="T21" s="30">
-        <f>ROUND(月別予算!$E$16*0.45,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="29" t="inlineStr">
-        <is>
-          <t>NORRONA STORE</t>
-        </is>
-      </c>
-      <c r="B22" s="29" t="inlineStr">
-        <is>
-          <t>ストア全体</t>
-        </is>
-      </c>
-      <c r="C22" s="29" t="inlineStr">
-        <is>
-          <t>Google</t>
-        </is>
-      </c>
-      <c r="D22" s="29" t="inlineStr">
-        <is>
-          <t>【新設】ショッピング(通常価格のみ)</t>
-        </is>
-      </c>
-      <c r="E22" s="30">
-        <f>ROUND(M22/30,-2)</f>
-        <v/>
-      </c>
-      <c r="F22" s="30">
-        <f>ROUND(N22/31,-2)</f>
-        <v/>
-      </c>
-      <c r="G22" s="30">
-        <f>ROUND(O22/30,-2)</f>
-        <v/>
-      </c>
-      <c r="H22" s="30">
-        <f>ROUND(P22/31,-2)</f>
-        <v/>
-      </c>
-      <c r="I22" s="30">
-        <f>ROUND(Q22/31,-2)</f>
-        <v/>
-      </c>
-      <c r="J22" s="30">
-        <f>ROUND(R22/28,-2)</f>
-        <v/>
-      </c>
-      <c r="K22" s="30">
-        <f>ROUND(S22/31,-2)</f>
-        <v/>
-      </c>
-      <c r="L22" s="30">
-        <f>ROUND(T22/30,-2)</f>
-        <v/>
-      </c>
-      <c r="M22" s="30">
-        <f>ROUND(月別予算!$E$9*0.3,0)</f>
-        <v/>
-      </c>
-      <c r="N22" s="30">
-        <f>ROUND(月別予算!$E$10*0.3,0)</f>
-        <v/>
-      </c>
-      <c r="O22" s="30">
-        <f>ROUND(月別予算!$E$11*0.3,0)</f>
-        <v/>
-      </c>
-      <c r="P22" s="30">
-        <f>ROUND(月別予算!$E$12*0.3,0)</f>
-        <v/>
-      </c>
-      <c r="Q22" s="30">
-        <f>ROUND(月別予算!$E$13*0.3,0)</f>
-        <v/>
-      </c>
-      <c r="R22" s="30">
-        <f>ROUND(月別予算!$E$14*0.3,0)</f>
-        <v/>
-      </c>
-      <c r="S22" s="30">
-        <f>ROUND(月別予算!$E$15*0.3,0)</f>
-        <v/>
-      </c>
-      <c r="T22" s="30">
-        <f>ROUND(月別予算!$E$16*0.3,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="29" t="inlineStr">
-        <is>
-          <t>NORRONA STORE</t>
-        </is>
-      </c>
-      <c r="B23" s="29" t="inlineStr">
-        <is>
-          <t>ストア全体</t>
-        </is>
-      </c>
-      <c r="C23" s="29" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
-      <c r="D23" s="29" t="inlineStr">
-        <is>
-          <t>【新設】カタログ/リターゲティング</t>
-        </is>
-      </c>
-      <c r="E23" s="30">
-        <f>ROUND(M23/30,-2)</f>
-        <v/>
-      </c>
-      <c r="F23" s="30">
-        <f>ROUND(N23/31,-2)</f>
-        <v/>
-      </c>
-      <c r="G23" s="30">
-        <f>ROUND(O23/30,-2)</f>
-        <v/>
-      </c>
-      <c r="H23" s="30">
-        <f>ROUND(P23/31,-2)</f>
-        <v/>
-      </c>
-      <c r="I23" s="30">
-        <f>ROUND(Q23/31,-2)</f>
-        <v/>
-      </c>
-      <c r="J23" s="30">
-        <f>ROUND(R23/28,-2)</f>
-        <v/>
-      </c>
-      <c r="K23" s="30">
-        <f>ROUND(S23/31,-2)</f>
-        <v/>
-      </c>
-      <c r="L23" s="30">
-        <f>ROUND(T23/30,-2)</f>
-        <v/>
-      </c>
-      <c r="M23" s="30">
-        <f>ROUND(月別予算!$E$9*0.25,0)</f>
-        <v/>
-      </c>
-      <c r="N23" s="30">
-        <f>ROUND(月別予算!$E$10*0.25,0)</f>
-        <v/>
-      </c>
-      <c r="O23" s="30">
-        <f>ROUND(月別予算!$E$11*0.25,0)</f>
-        <v/>
-      </c>
-      <c r="P23" s="30">
-        <f>ROUND(月別予算!$E$12*0.25,0)</f>
-        <v/>
-      </c>
-      <c r="Q23" s="30">
-        <f>ROUND(月別予算!$E$13*0.25,0)</f>
-        <v/>
-      </c>
-      <c r="R23" s="30">
-        <f>ROUND(月別予算!$E$14*0.25,0)</f>
-        <v/>
-      </c>
-      <c r="S23" s="30">
-        <f>ROUND(月別予算!$E$15*0.25,0)</f>
-        <v/>
-      </c>
-      <c r="T23" s="30">
-        <f>ROUND(月別予算!$E$16*0.25,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="29" t="inlineStr">
-        <is>
-          <t>PU STORE</t>
-        </is>
-      </c>
-      <c r="B24" s="29" t="inlineStr">
-        <is>
-          <t>ストア全体</t>
-        </is>
-      </c>
-      <c r="C24" s="29" t="inlineStr">
-        <is>
-          <t>Google</t>
-        </is>
-      </c>
-      <c r="D24" s="29" t="inlineStr">
-        <is>
-          <t>【新設】指名検索</t>
-        </is>
-      </c>
-      <c r="E24" s="30">
-        <f>ROUND(M24/30,-2)</f>
-        <v/>
-      </c>
-      <c r="F24" s="30">
-        <f>ROUND(N24/31,-2)</f>
-        <v/>
-      </c>
-      <c r="G24" s="30">
-        <f>ROUND(O24/30,-2)</f>
-        <v/>
-      </c>
-      <c r="H24" s="30">
-        <f>ROUND(P24/31,-2)</f>
-        <v/>
-      </c>
-      <c r="I24" s="30">
-        <f>ROUND(Q24/31,-2)</f>
-        <v/>
-      </c>
-      <c r="J24" s="30">
-        <f>ROUND(R24/28,-2)</f>
-        <v/>
-      </c>
-      <c r="K24" s="30">
-        <f>ROUND(S24/31,-2)</f>
-        <v/>
-      </c>
-      <c r="L24" s="30">
-        <f>ROUND(T24/30,-2)</f>
-        <v/>
-      </c>
-      <c r="M24" s="30">
-        <f>ROUND(月別予算!$F$9*0.45,0)</f>
-        <v/>
-      </c>
-      <c r="N24" s="30">
-        <f>ROUND(月別予算!$F$10*0.45,0)</f>
-        <v/>
-      </c>
-      <c r="O24" s="30">
-        <f>ROUND(月別予算!$F$11*0.45,0)</f>
-        <v/>
-      </c>
-      <c r="P24" s="30">
-        <f>ROUND(月別予算!$F$12*0.45,0)</f>
-        <v/>
-      </c>
-      <c r="Q24" s="30">
-        <f>ROUND(月別予算!$F$13*0.45,0)</f>
-        <v/>
-      </c>
-      <c r="R24" s="30">
-        <f>ROUND(月別予算!$F$14*0.45,0)</f>
-        <v/>
-      </c>
-      <c r="S24" s="30">
-        <f>ROUND(月別予算!$F$15*0.45,0)</f>
-        <v/>
-      </c>
-      <c r="T24" s="30">
-        <f>ROUND(月別予算!$F$16*0.45,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="29" t="inlineStr">
-        <is>
-          <t>PU STORE</t>
-        </is>
-      </c>
-      <c r="B25" s="29" t="inlineStr">
-        <is>
-          <t>ストア全体</t>
-        </is>
-      </c>
-      <c r="C25" s="29" t="inlineStr">
-        <is>
-          <t>Google</t>
-        </is>
-      </c>
-      <c r="D25" s="29" t="inlineStr">
-        <is>
-          <t>【新設】ショッピング(通常価格のみ)</t>
-        </is>
-      </c>
-      <c r="E25" s="30">
-        <f>ROUND(M25/30,-2)</f>
-        <v/>
-      </c>
-      <c r="F25" s="30">
-        <f>ROUND(N25/31,-2)</f>
-        <v/>
-      </c>
-      <c r="G25" s="30">
-        <f>ROUND(O25/30,-2)</f>
-        <v/>
-      </c>
-      <c r="H25" s="30">
-        <f>ROUND(P25/31,-2)</f>
-        <v/>
-      </c>
-      <c r="I25" s="30">
-        <f>ROUND(Q25/31,-2)</f>
-        <v/>
-      </c>
-      <c r="J25" s="30">
-        <f>ROUND(R25/28,-2)</f>
-        <v/>
-      </c>
-      <c r="K25" s="30">
-        <f>ROUND(S25/31,-2)</f>
-        <v/>
-      </c>
-      <c r="L25" s="30">
-        <f>ROUND(T25/30,-2)</f>
-        <v/>
-      </c>
-      <c r="M25" s="30">
-        <f>ROUND(月別予算!$F$9*0.3,0)</f>
-        <v/>
-      </c>
-      <c r="N25" s="30">
-        <f>ROUND(月別予算!$F$10*0.3,0)</f>
-        <v/>
-      </c>
-      <c r="O25" s="30">
-        <f>ROUND(月別予算!$F$11*0.3,0)</f>
-        <v/>
-      </c>
-      <c r="P25" s="30">
-        <f>ROUND(月別予算!$F$12*0.3,0)</f>
-        <v/>
-      </c>
-      <c r="Q25" s="30">
-        <f>ROUND(月別予算!$F$13*0.3,0)</f>
-        <v/>
-      </c>
-      <c r="R25" s="30">
-        <f>ROUND(月別予算!$F$14*0.3,0)</f>
-        <v/>
-      </c>
-      <c r="S25" s="30">
-        <f>ROUND(月別予算!$F$15*0.3,0)</f>
-        <v/>
-      </c>
-      <c r="T25" s="30">
-        <f>ROUND(月別予算!$F$16*0.3,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="29" t="inlineStr">
-        <is>
-          <t>PU STORE</t>
-        </is>
-      </c>
-      <c r="B26" s="29" t="inlineStr">
-        <is>
-          <t>ストア全体</t>
-        </is>
-      </c>
-      <c r="C26" s="29" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
-      <c r="D26" s="29" t="inlineStr">
-        <is>
-          <t>【新設】カタログ/リターゲティング</t>
-        </is>
-      </c>
-      <c r="E26" s="30">
-        <f>ROUND(M26/30,-2)</f>
-        <v/>
-      </c>
-      <c r="F26" s="30">
-        <f>ROUND(N26/31,-2)</f>
-        <v/>
-      </c>
-      <c r="G26" s="30">
-        <f>ROUND(O26/30,-2)</f>
-        <v/>
-      </c>
-      <c r="H26" s="30">
-        <f>ROUND(P26/31,-2)</f>
-        <v/>
-      </c>
-      <c r="I26" s="30">
-        <f>ROUND(Q26/31,-2)</f>
-        <v/>
-      </c>
-      <c r="J26" s="30">
-        <f>ROUND(R26/28,-2)</f>
-        <v/>
-      </c>
-      <c r="K26" s="30">
-        <f>ROUND(S26/31,-2)</f>
-        <v/>
-      </c>
-      <c r="L26" s="30">
-        <f>ROUND(T26/30,-2)</f>
-        <v/>
-      </c>
-      <c r="M26" s="30">
-        <f>ROUND(月別予算!$F$9*0.25,0)</f>
-        <v/>
-      </c>
-      <c r="N26" s="30">
-        <f>ROUND(月別予算!$F$10*0.25,0)</f>
-        <v/>
-      </c>
-      <c r="O26" s="30">
-        <f>ROUND(月別予算!$F$11*0.25,0)</f>
-        <v/>
-      </c>
-      <c r="P26" s="30">
-        <f>ROUND(月別予算!$F$12*0.25,0)</f>
-        <v/>
-      </c>
-      <c r="Q26" s="30">
-        <f>ROUND(月別予算!$F$13*0.25,0)</f>
-        <v/>
-      </c>
-      <c r="R26" s="30">
-        <f>ROUND(月別予算!$F$14*0.25,0)</f>
-        <v/>
-      </c>
-      <c r="S26" s="30">
-        <f>ROUND(月別予算!$F$15*0.25,0)</f>
-        <v/>
-      </c>
-      <c r="T26" s="30">
-        <f>ROUND(月別予算!$F$16*0.25,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="21" t="inlineStr">
-        <is>
-          <t>合計（通常運用）</t>
-        </is>
-      </c>
-      <c r="B27" s="18" t="n"/>
-      <c r="C27" s="18" t="n"/>
-      <c r="D27" s="18" t="n"/>
-      <c r="E27" s="22">
-        <f>SUM(E4:E26)</f>
-        <v/>
-      </c>
-      <c r="F27" s="22">
-        <f>SUM(F4:F26)</f>
-        <v/>
-      </c>
-      <c r="G27" s="22">
-        <f>SUM(G4:G26)</f>
-        <v/>
-      </c>
-      <c r="H27" s="22">
-        <f>SUM(H4:H26)</f>
-        <v/>
-      </c>
-      <c r="I27" s="22">
-        <f>SUM(I4:I26)</f>
-        <v/>
-      </c>
-      <c r="J27" s="22">
-        <f>SUM(J4:J26)</f>
-        <v/>
-      </c>
-      <c r="K27" s="22">
-        <f>SUM(K4:K26)</f>
-        <v/>
-      </c>
-      <c r="L27" s="22">
-        <f>SUM(L4:L26)</f>
-        <v/>
-      </c>
-      <c r="M27" s="22">
-        <f>SUM(M4:M26)</f>
-        <v/>
-      </c>
-      <c r="N27" s="22">
-        <f>SUM(N4:N26)</f>
-        <v/>
-      </c>
-      <c r="O27" s="22">
-        <f>SUM(O4:O26)</f>
-        <v/>
-      </c>
-      <c r="P27" s="22">
-        <f>SUM(P4:P26)</f>
-        <v/>
-      </c>
-      <c r="Q27" s="22">
-        <f>SUM(Q4:Q26)</f>
-        <v/>
-      </c>
-      <c r="R27" s="22">
-        <f>SUM(R4:R26)</f>
-        <v/>
-      </c>
-      <c r="S27" s="22">
-        <f>SUM(S4:S26)</f>
-        <v/>
-      </c>
-      <c r="T27" s="22">
-        <f>SUM(T4:T26)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="21" t="inlineStr">
+      <c r="A19" s="21" t="inlineStr">
         <is>
           <t>イベント予備費（別枠）</t>
         </is>
       </c>
-      <c r="B28" s="18" t="n"/>
-      <c r="C28" s="18" t="n"/>
-      <c r="D28" s="18" t="n"/>
-      <c r="E28" s="18" t="n"/>
-      <c r="F28" s="18" t="n"/>
-      <c r="G28" s="18" t="n"/>
-      <c r="H28" s="18" t="n"/>
-      <c r="I28" s="18" t="n"/>
-      <c r="J28" s="18" t="n"/>
-      <c r="K28" s="18" t="n"/>
-      <c r="L28" s="18" t="n"/>
-      <c r="M28" s="19">
+      <c r="B19" s="18" t="n"/>
+      <c r="C19" s="18" t="n"/>
+      <c r="D19" s="18" t="n"/>
+      <c r="E19" s="18" t="n"/>
+      <c r="F19" s="18" t="n"/>
+      <c r="G19" s="18" t="n"/>
+      <c r="H19" s="18" t="n"/>
+      <c r="I19" s="18" t="n"/>
+      <c r="J19" s="18" t="n"/>
+      <c r="K19" s="18" t="n"/>
+      <c r="L19" s="18" t="n"/>
+      <c r="M19" s="19">
         <f>月別予算!$I$9</f>
         <v/>
       </c>
-      <c r="N28" s="19">
+      <c r="N19" s="19">
         <f>月別予算!$I$10</f>
         <v/>
       </c>
-      <c r="O28" s="19">
+      <c r="O19" s="19">
         <f>月別予算!$I$11</f>
         <v/>
       </c>
-      <c r="P28" s="19">
+      <c r="P19" s="19">
         <f>月別予算!$I$12</f>
         <v/>
       </c>
-      <c r="Q28" s="19">
+      <c r="Q19" s="19">
         <f>月別予算!$I$13</f>
         <v/>
       </c>
-      <c r="R28" s="19">
+      <c r="R19" s="19">
         <f>月別予算!$I$14</f>
         <v/>
       </c>
-      <c r="S28" s="19">
+      <c r="S19" s="19">
         <f>月別予算!$I$15</f>
         <v/>
       </c>
-      <c r="T28" s="19">
+      <c r="T19" s="19">
         <f>月別予算!$I$16</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Rebuild October budget: ~800k yen, shift the rest to Nov-Dec winter items
October normal operations drop to 800,286 yen; Nov/Dec gain 150k/100k for
regular-price winter items (event reserves unchanged). Adds a campaign-level
October daily budget plan and scripts/apply_budget_plan.py to preview or
apply it after approval.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EFkMa7pBd48FUqtUrcDcW8
</commit_message>
<xml_diff>
--- a/reports/広告予算計画_2026-09改訂.xlsx
+++ b/reports/広告予算計画_2026-09改訂.xlsx
@@ -886,7 +886,7 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>0.15</v>
+        <v>0.1141</v>
       </c>
     </row>
     <row r="29">
@@ -896,7 +896,7 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>0.155</v>
+        <v>0.1764</v>
       </c>
     </row>
     <row r="30">
@@ -906,7 +906,7 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>0.17</v>
+        <v>0.1846</v>
       </c>
     </row>
     <row r="31">
@@ -1100,11 +1100,11 @@
         <v>0.05</v>
       </c>
       <c r="C45" s="5" t="n">
-        <v>0.05</v>
+        <v>0.03</v>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>ユーザー判断で維持（売れる見込み）</t>
+          <t>8〜9月の売上の72%がセール品、広告 ROAS 2.6。縮小</t>
         </is>
       </c>
     </row>
@@ -1118,11 +1118,11 @@
         <v>0.04</v>
       </c>
       <c r="C46" s="5" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>10〜1月が本番。フィード未掲載の解消が前提</t>
+          <t>10〜1月が本番。売上の79%が通常品（粗利50%）。フィード未掲載の解消が前提</t>
         </is>
       </c>
     </row>
@@ -1603,7 +1603,7 @@
       </c>
       <c r="M10" s="17" t="inlineStr">
         <is>
-          <t>勝負月</t>
+          <t>冬物の立ち上がり前。約80万に抑え、11〜12月の通常品の冬物へ回す</t>
         </is>
       </c>
     </row>
@@ -2364,7 +2364,7 @@
       </c>
       <c r="K10" s="17" t="inlineStr">
         <is>
-          <t>ユーザー判断で維持（売れる見込み）</t>
+          <t>8〜9月の売上の72%がセール品、広告 ROAS 2.6。縮小</t>
         </is>
       </c>
     </row>
@@ -2412,7 +2412,7 @@
       </c>
       <c r="K11" s="17" t="inlineStr">
         <is>
-          <t>10〜1月が本番。フィード未掲載の解消が前提</t>
+          <t>10〜1月が本番。売上の79%が通常品（粗利50%）。フィード未掲載の解消が前提</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add a 100k yen Black Friday event reserve (moved from November normal budget)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EFkMa7pBd48FUqtUrcDcW8
</commit_message>
<xml_diff>
--- a/reports/広告予算計画_2026-09改訂.xlsx
+++ b/reports/広告予算計画_2026-09改訂.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -807,12 +807,12 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>2026-12</t>
+          <t>2026-11</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>年末年始企画</t>
+          <t>ブラックフライデー（他社と同日程・約4日間。11月の通常運用から10万を移す）</t>
         </is>
       </c>
       <c r="C21" s="12" t="n">
@@ -822,332 +822,329 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>2027-02</t>
+          <t>2026-12</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>冬セール</t>
+          <t>年末年始企画</t>
         </is>
       </c>
       <c r="C22" s="12" t="n">
-        <v>250000</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
+          <t>2027-02</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>冬セール</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="n">
+        <v>250000</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
           <t>2027-03</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>イベント告知予備</t>
         </is>
       </c>
-      <c r="C23" s="12" t="n">
+      <c r="C24" s="12" t="n">
         <v>50000</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="7" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
         <is>
           <t>計</t>
         </is>
       </c>
-      <c r="C24" s="8">
-        <f>SUM(C20:C23)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="7" t="inlineStr">
+      <c r="C25" s="8">
+        <f>SUM(C20:C24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
         <is>
           <t>10〜4月 通常運用の月別配分比率（繁忙期に厚く。4月は残額調整）</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="9" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr">
         <is>
           <t>月</t>
         </is>
       </c>
-      <c r="B27" s="9" t="inlineStr">
+      <c r="B28" s="9" t="inlineStr">
         <is>
           <t>比率</t>
         </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>2026-10</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="n">
-        <v>0.1141</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>2026-11</t>
+          <t>2026-10</t>
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>0.1764</v>
+        <v>0.11575</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>2026-12</t>
+          <t>2026-11</t>
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>0.1846</v>
+        <v>0.16449</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>2027-01</t>
+          <t>2026-12</t>
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>0.14</v>
+        <v>0.18727</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>2027-02</t>
+          <t>2027-01</t>
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>0.16</v>
+        <v>0.14203</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>2027-03</t>
+          <t>2027-02</t>
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>0.115</v>
+        <v>0.16231</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
+          <t>2027-03</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>0.11666</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
           <t>2027-04</t>
         </is>
       </c>
-      <c r="B34" s="5" t="n">
+      <c r="B35" s="5" t="n">
         <v>0.11</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="7" t="inlineStr">
-        <is>
-          <t>計（100%）</t>
-        </is>
-      </c>
-      <c r="B35" s="13">
-        <f>SUM(B28:B34)</f>
-        <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
+          <t>計（100%）</t>
+        </is>
+      </c>
+      <c r="B36" s="13">
+        <f>SUM(B29:B35)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
           <t>10〜4月 通常運用の総額（上限−実績−9月−イベント）</t>
         </is>
       </c>
-      <c r="B36" s="8">
-        <f>前提!$B$8-前提!$D$15-前提!$B$6-前提!$C$24</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="7" t="inlineStr">
+      <c r="B37" s="8">
+        <f>前提!$B$8-前提!$D$15-前提!$B$6-前提!$C$25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="7" t="inlineStr">
         <is>
           <t>FULLMARKS 内のブランド配分比率</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="9" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="9" t="inlineStr">
         <is>
           <t>ブランド/枠</t>
         </is>
       </c>
-      <c r="B39" s="9" t="inlineStr">
+      <c r="B40" s="9" t="inlineStr">
         <is>
           <t>9月 比率</t>
         </is>
       </c>
-      <c r="C39" s="9" t="inlineStr">
+      <c r="C40" s="9" t="inlineStr">
         <is>
           <t>10月〜 比率</t>
         </is>
       </c>
-      <c r="D39" s="9" t="inlineStr">
+      <c r="D40" s="9" t="inlineStr">
         <is>
           <t>備考</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="3" t="inlineStr">
-        <is>
-          <t>HOUDINI</t>
-        </is>
-      </c>
-      <c r="B40" s="5" t="n">
-        <v>0.27</v>
-      </c>
-      <c r="C40" s="5" t="n">
-        <v>0.26</v>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>広告売上の半分以上（9月 ROAS 11.8）。FULLMARKS で継続</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>商品連動(ショッピング/カタログ)</t>
+          <t>HOUDINI</t>
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>0.3</v>
+        <v>0.27</v>
       </c>
       <c r="C41" s="5" t="n">
-        <v>0.23</v>
+        <v>0.26</v>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>通常価格品のみ（アウトレットは広告しない）。9月 ROAS: カタログ 4.6 / ショッピング 2.5。ショッピングを絞る</t>
+          <t>広告売上の半分以上（9月 ROAS 11.8）。FULLMARKS で継続</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>店舗指名(フルマークス)</t>
+          <t>商品連動(ショッピング/カタログ)</t>
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>0.17</v>
+        <v>0.3</v>
       </c>
       <c r="C42" s="5" t="n">
-        <v>0.18</v>
+        <v>0.23</v>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>9月 ROAS 16.2 の安定枠</t>
+          <t>通常価格品のみ（アウトレットは広告しない）。9月 ROAS: カタログ 4.6 / ショッピング 2.5。ショッピングを絞る</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>POC</t>
+          <t>店舗指名(フルマークス)</t>
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>0.09</v>
+        <v>0.17</v>
       </c>
       <c r="C43" s="5" t="n">
-        <v>0.11</v>
+        <v>0.18</v>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>9月 ROAS 3.8。10月以降やや厚く</t>
+          <t>9月 ROAS 16.2 の安定枠</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>NORRØNA</t>
+          <t>POC</t>
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.09</v>
       </c>
       <c r="C44" s="5" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.11</v>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>9月 ROAS 4.1（8月 1.0 から改善）。FULLMARKS で継続</t>
+          <t>9月 ROAS 3.8。10月以降やや厚く</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>ACLIMA</t>
+          <t>NORRØNA</t>
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>0.05</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="C45" s="5" t="n">
-        <v>0.03</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>8〜9月の売上の72%がセール品、広告 ROAS 2.6。縮小</t>
+          <t>9月 ROAS 4.1（8月 1.0 から改善）。FULLMARKS で継続</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>HESTRA【新規】</t>
+          <t>ACLIMA</t>
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="C46" s="5" t="n">
-        <v>0.1</v>
+        <v>0.03</v>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>10〜1月が本番。売上の79%が通常品（粗利50%）。フィード未掲載の解消が前提</t>
+          <t>8〜9月の売上の72%がセール品、広告 ROAS 2.6。縮小</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>KANG【新規】</t>
+          <t>HESTRA【新規】</t>
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>0.005</v>
+        <v>0.04</v>
       </c>
       <c r="C47" s="5" t="n">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>テスト枠</t>
+          <t>10〜1月が本番。売上の79%が通常品（粗利50%）。フィード未掲載の解消が前提</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>PLUS ONE WORKS【新規】</t>
+          <t>KANG【新規】</t>
         </is>
       </c>
       <c r="B48" s="5" t="n">
@@ -1163,17 +1160,35 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="7" t="inlineStr">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>PLUS ONE WORKS【新規】</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="C49" s="5" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>テスト枠</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="7" t="inlineStr">
         <is>
           <t>計（各100%）</t>
         </is>
       </c>
-      <c r="B49" s="13">
-        <f>SUM(B40:B48)</f>
-        <v/>
-      </c>
-      <c r="C49" s="13">
-        <f>SUM(C40:C48)</f>
+      <c r="B50" s="13">
+        <f>SUM(B41:B49)</f>
+        <v/>
+      </c>
+      <c r="C50" s="13">
+        <f>SUM(C41:C49)</f>
         <v/>
       </c>
     </row>
@@ -1583,7 +1598,7 @@
         <v>0</v>
       </c>
       <c r="H10" s="20">
-        <f>前提!$B$36*前提!$B$28</f>
+        <f>前提!$B$37*前提!$B$29</f>
         <v/>
       </c>
       <c r="I10" s="20" t="n">
@@ -1638,11 +1653,12 @@
         <v>0</v>
       </c>
       <c r="H11" s="20">
-        <f>前提!$B$36*前提!$B$29</f>
-        <v/>
-      </c>
-      <c r="I11" s="20" t="n">
-        <v>0</v>
+        <f>前提!$B$37*前提!$B$30</f>
+        <v/>
+      </c>
+      <c r="I11" s="19">
+        <f>前提!C21</f>
+        <v/>
       </c>
       <c r="J11" s="20">
         <f>H11+I11</f>
@@ -1689,11 +1705,11 @@
         <v>0</v>
       </c>
       <c r="H12" s="20">
-        <f>前提!$B$36*前提!$B$30</f>
+        <f>前提!$B$37*前提!$B$31</f>
         <v/>
       </c>
       <c r="I12" s="19">
-        <f>前提!C21</f>
+        <f>前提!C22</f>
         <v/>
       </c>
       <c r="J12" s="20">
@@ -1745,7 +1761,7 @@
         <v>0</v>
       </c>
       <c r="H13" s="20">
-        <f>前提!$B$36*前提!$B$31</f>
+        <f>前提!$B$37*前提!$B$32</f>
         <v/>
       </c>
       <c r="I13" s="20" t="n">
@@ -1796,11 +1812,11 @@
         <v>0</v>
       </c>
       <c r="H14" s="20">
-        <f>前提!$B$36*前提!$B$32</f>
+        <f>前提!$B$37*前提!$B$33</f>
         <v/>
       </c>
       <c r="I14" s="19">
-        <f>前提!C22</f>
+        <f>前提!C23</f>
         <v/>
       </c>
       <c r="J14" s="20">
@@ -1852,11 +1868,11 @@
         <v>0</v>
       </c>
       <c r="H15" s="20">
-        <f>前提!$B$36*前提!$B$33</f>
+        <f>前提!$B$37*前提!$B$34</f>
         <v/>
       </c>
       <c r="I15" s="19">
-        <f>前提!C23</f>
+        <f>前提!C24</f>
         <v/>
       </c>
       <c r="J15" s="20">
@@ -1908,7 +1924,7 @@
         <v>0</v>
       </c>
       <c r="H16" s="20">
-        <f>前提!$B$36-SUM(H10:H15)</f>
+        <f>前提!$B$37-SUM(H10:H15)</f>
         <v/>
       </c>
       <c r="I16" s="20" t="n">
@@ -2087,35 +2103,35 @@
         </is>
       </c>
       <c r="B5" s="19">
-        <f>ROUND(月別予算!$C$9*前提!$B$40,0)</f>
+        <f>ROUND(月別予算!$C$9*前提!$B$41,0)</f>
         <v/>
       </c>
       <c r="C5" s="19">
-        <f>ROUND(月別予算!$C$10*前提!$C$40,0)</f>
+        <f>ROUND(月別予算!$C$10*前提!$C$41,0)</f>
         <v/>
       </c>
       <c r="D5" s="19">
-        <f>ROUND(月別予算!$C$11*前提!$C$40,0)</f>
+        <f>ROUND(月別予算!$C$11*前提!$C$41,0)</f>
         <v/>
       </c>
       <c r="E5" s="19">
-        <f>ROUND(月別予算!$C$12*前提!$C$40,0)</f>
+        <f>ROUND(月別予算!$C$12*前提!$C$41,0)</f>
         <v/>
       </c>
       <c r="F5" s="19">
-        <f>ROUND(月別予算!$C$13*前提!$C$40,0)</f>
+        <f>ROUND(月別予算!$C$13*前提!$C$41,0)</f>
         <v/>
       </c>
       <c r="G5" s="19">
-        <f>ROUND(月別予算!$C$14*前提!$C$40,0)</f>
+        <f>ROUND(月別予算!$C$14*前提!$C$41,0)</f>
         <v/>
       </c>
       <c r="H5" s="19">
-        <f>ROUND(月別予算!$C$15*前提!$C$40,0)</f>
+        <f>ROUND(月別予算!$C$15*前提!$C$41,0)</f>
         <v/>
       </c>
       <c r="I5" s="19">
-        <f>ROUND(月別予算!$C$16*前提!$C$40,0)</f>
+        <f>ROUND(月別予算!$C$16*前提!$C$41,0)</f>
         <v/>
       </c>
       <c r="J5" s="23">
@@ -2135,35 +2151,35 @@
         </is>
       </c>
       <c r="B6" s="19">
-        <f>ROUND(月別予算!$C$9*前提!$B$41,0)</f>
+        <f>ROUND(月別予算!$C$9*前提!$B$42,0)</f>
         <v/>
       </c>
       <c r="C6" s="19">
-        <f>ROUND(月別予算!$C$10*前提!$C$41,0)</f>
+        <f>ROUND(月別予算!$C$10*前提!$C$42,0)</f>
         <v/>
       </c>
       <c r="D6" s="19">
-        <f>ROUND(月別予算!$C$11*前提!$C$41,0)</f>
+        <f>ROUND(月別予算!$C$11*前提!$C$42,0)</f>
         <v/>
       </c>
       <c r="E6" s="19">
-        <f>ROUND(月別予算!$C$12*前提!$C$41,0)</f>
+        <f>ROUND(月別予算!$C$12*前提!$C$42,0)</f>
         <v/>
       </c>
       <c r="F6" s="19">
-        <f>ROUND(月別予算!$C$13*前提!$C$41,0)</f>
+        <f>ROUND(月別予算!$C$13*前提!$C$42,0)</f>
         <v/>
       </c>
       <c r="G6" s="19">
-        <f>ROUND(月別予算!$C$14*前提!$C$41,0)</f>
+        <f>ROUND(月別予算!$C$14*前提!$C$42,0)</f>
         <v/>
       </c>
       <c r="H6" s="19">
-        <f>ROUND(月別予算!$C$15*前提!$C$41,0)</f>
+        <f>ROUND(月別予算!$C$15*前提!$C$42,0)</f>
         <v/>
       </c>
       <c r="I6" s="19">
-        <f>ROUND(月別予算!$C$16*前提!$C$41,0)</f>
+        <f>ROUND(月別予算!$C$16*前提!$C$42,0)</f>
         <v/>
       </c>
       <c r="J6" s="23">
@@ -2183,35 +2199,35 @@
         </is>
       </c>
       <c r="B7" s="19">
-        <f>ROUND(月別予算!$C$9*前提!$B$42,0)</f>
+        <f>ROUND(月別予算!$C$9*前提!$B$43,0)</f>
         <v/>
       </c>
       <c r="C7" s="19">
-        <f>ROUND(月別予算!$C$10*前提!$C$42,0)</f>
+        <f>ROUND(月別予算!$C$10*前提!$C$43,0)</f>
         <v/>
       </c>
       <c r="D7" s="19">
-        <f>ROUND(月別予算!$C$11*前提!$C$42,0)</f>
+        <f>ROUND(月別予算!$C$11*前提!$C$43,0)</f>
         <v/>
       </c>
       <c r="E7" s="19">
-        <f>ROUND(月別予算!$C$12*前提!$C$42,0)</f>
+        <f>ROUND(月別予算!$C$12*前提!$C$43,0)</f>
         <v/>
       </c>
       <c r="F7" s="19">
-        <f>ROUND(月別予算!$C$13*前提!$C$42,0)</f>
+        <f>ROUND(月別予算!$C$13*前提!$C$43,0)</f>
         <v/>
       </c>
       <c r="G7" s="19">
-        <f>ROUND(月別予算!$C$14*前提!$C$42,0)</f>
+        <f>ROUND(月別予算!$C$14*前提!$C$43,0)</f>
         <v/>
       </c>
       <c r="H7" s="19">
-        <f>ROUND(月別予算!$C$15*前提!$C$42,0)</f>
+        <f>ROUND(月別予算!$C$15*前提!$C$43,0)</f>
         <v/>
       </c>
       <c r="I7" s="19">
-        <f>ROUND(月別予算!$C$16*前提!$C$42,0)</f>
+        <f>ROUND(月別予算!$C$16*前提!$C$43,0)</f>
         <v/>
       </c>
       <c r="J7" s="23">
@@ -2231,35 +2247,35 @@
         </is>
       </c>
       <c r="B8" s="19">
-        <f>ROUND(月別予算!$C$9*前提!$B$43,0)</f>
+        <f>ROUND(月別予算!$C$9*前提!$B$44,0)</f>
         <v/>
       </c>
       <c r="C8" s="19">
-        <f>ROUND(月別予算!$C$10*前提!$C$43,0)</f>
+        <f>ROUND(月別予算!$C$10*前提!$C$44,0)</f>
         <v/>
       </c>
       <c r="D8" s="19">
-        <f>ROUND(月別予算!$C$11*前提!$C$43,0)</f>
+        <f>ROUND(月別予算!$C$11*前提!$C$44,0)</f>
         <v/>
       </c>
       <c r="E8" s="19">
-        <f>ROUND(月別予算!$C$12*前提!$C$43,0)</f>
+        <f>ROUND(月別予算!$C$12*前提!$C$44,0)</f>
         <v/>
       </c>
       <c r="F8" s="19">
-        <f>ROUND(月別予算!$C$13*前提!$C$43,0)</f>
+        <f>ROUND(月別予算!$C$13*前提!$C$44,0)</f>
         <v/>
       </c>
       <c r="G8" s="19">
-        <f>ROUND(月別予算!$C$14*前提!$C$43,0)</f>
+        <f>ROUND(月別予算!$C$14*前提!$C$44,0)</f>
         <v/>
       </c>
       <c r="H8" s="19">
-        <f>ROUND(月別予算!$C$15*前提!$C$43,0)</f>
+        <f>ROUND(月別予算!$C$15*前提!$C$44,0)</f>
         <v/>
       </c>
       <c r="I8" s="19">
-        <f>ROUND(月別予算!$C$16*前提!$C$43,0)</f>
+        <f>ROUND(月別予算!$C$16*前提!$C$44,0)</f>
         <v/>
       </c>
       <c r="J8" s="23">
@@ -2279,35 +2295,35 @@
         </is>
       </c>
       <c r="B9" s="19">
-        <f>ROUND(月別予算!$C$9*前提!$B$44,0)</f>
+        <f>ROUND(月別予算!$C$9*前提!$B$45,0)</f>
         <v/>
       </c>
       <c r="C9" s="19">
-        <f>ROUND(月別予算!$C$10*前提!$C$44,0)</f>
+        <f>ROUND(月別予算!$C$10*前提!$C$45,0)</f>
         <v/>
       </c>
       <c r="D9" s="19">
-        <f>ROUND(月別予算!$C$11*前提!$C$44,0)</f>
+        <f>ROUND(月別予算!$C$11*前提!$C$45,0)</f>
         <v/>
       </c>
       <c r="E9" s="19">
-        <f>ROUND(月別予算!$C$12*前提!$C$44,0)</f>
+        <f>ROUND(月別予算!$C$12*前提!$C$45,0)</f>
         <v/>
       </c>
       <c r="F9" s="19">
-        <f>ROUND(月別予算!$C$13*前提!$C$44,0)</f>
+        <f>ROUND(月別予算!$C$13*前提!$C$45,0)</f>
         <v/>
       </c>
       <c r="G9" s="19">
-        <f>ROUND(月別予算!$C$14*前提!$C$44,0)</f>
+        <f>ROUND(月別予算!$C$14*前提!$C$45,0)</f>
         <v/>
       </c>
       <c r="H9" s="19">
-        <f>ROUND(月別予算!$C$15*前提!$C$44,0)</f>
+        <f>ROUND(月別予算!$C$15*前提!$C$45,0)</f>
         <v/>
       </c>
       <c r="I9" s="19">
-        <f>ROUND(月別予算!$C$16*前提!$C$44,0)</f>
+        <f>ROUND(月別予算!$C$16*前提!$C$45,0)</f>
         <v/>
       </c>
       <c r="J9" s="23">
@@ -2327,35 +2343,35 @@
         </is>
       </c>
       <c r="B10" s="19">
-        <f>ROUND(月別予算!$C$9*前提!$B$45,0)</f>
+        <f>ROUND(月別予算!$C$9*前提!$B$46,0)</f>
         <v/>
       </c>
       <c r="C10" s="19">
-        <f>ROUND(月別予算!$C$10*前提!$C$45,0)</f>
+        <f>ROUND(月別予算!$C$10*前提!$C$46,0)</f>
         <v/>
       </c>
       <c r="D10" s="19">
-        <f>ROUND(月別予算!$C$11*前提!$C$45,0)</f>
+        <f>ROUND(月別予算!$C$11*前提!$C$46,0)</f>
         <v/>
       </c>
       <c r="E10" s="19">
-        <f>ROUND(月別予算!$C$12*前提!$C$45,0)</f>
+        <f>ROUND(月別予算!$C$12*前提!$C$46,0)</f>
         <v/>
       </c>
       <c r="F10" s="19">
-        <f>ROUND(月別予算!$C$13*前提!$C$45,0)</f>
+        <f>ROUND(月別予算!$C$13*前提!$C$46,0)</f>
         <v/>
       </c>
       <c r="G10" s="19">
-        <f>ROUND(月別予算!$C$14*前提!$C$45,0)</f>
+        <f>ROUND(月別予算!$C$14*前提!$C$46,0)</f>
         <v/>
       </c>
       <c r="H10" s="19">
-        <f>ROUND(月別予算!$C$15*前提!$C$45,0)</f>
+        <f>ROUND(月別予算!$C$15*前提!$C$46,0)</f>
         <v/>
       </c>
       <c r="I10" s="19">
-        <f>ROUND(月別予算!$C$16*前提!$C$45,0)</f>
+        <f>ROUND(月別予算!$C$16*前提!$C$46,0)</f>
         <v/>
       </c>
       <c r="J10" s="23">
@@ -2375,35 +2391,35 @@
         </is>
       </c>
       <c r="B11" s="27">
-        <f>ROUND(月別予算!$C$9*前提!$B$46,0)</f>
+        <f>ROUND(月別予算!$C$9*前提!$B$47,0)</f>
         <v/>
       </c>
       <c r="C11" s="27">
-        <f>ROUND(月別予算!$C$10*前提!$C$46,0)</f>
+        <f>ROUND(月別予算!$C$10*前提!$C$47,0)</f>
         <v/>
       </c>
       <c r="D11" s="27">
-        <f>ROUND(月別予算!$C$11*前提!$C$46,0)</f>
+        <f>ROUND(月別予算!$C$11*前提!$C$47,0)</f>
         <v/>
       </c>
       <c r="E11" s="27">
-        <f>ROUND(月別予算!$C$12*前提!$C$46,0)</f>
+        <f>ROUND(月別予算!$C$12*前提!$C$47,0)</f>
         <v/>
       </c>
       <c r="F11" s="27">
-        <f>ROUND(月別予算!$C$13*前提!$C$46,0)</f>
+        <f>ROUND(月別予算!$C$13*前提!$C$47,0)</f>
         <v/>
       </c>
       <c r="G11" s="27">
-        <f>ROUND(月別予算!$C$14*前提!$C$46,0)</f>
+        <f>ROUND(月別予算!$C$14*前提!$C$47,0)</f>
         <v/>
       </c>
       <c r="H11" s="27">
-        <f>ROUND(月別予算!$C$15*前提!$C$46,0)</f>
+        <f>ROUND(月別予算!$C$15*前提!$C$47,0)</f>
         <v/>
       </c>
       <c r="I11" s="27">
-        <f>ROUND(月別予算!$C$16*前提!$C$46,0)</f>
+        <f>ROUND(月別予算!$C$16*前提!$C$47,0)</f>
         <v/>
       </c>
       <c r="J11" s="28">
@@ -2423,35 +2439,35 @@
         </is>
       </c>
       <c r="B12" s="27">
-        <f>ROUND(月別予算!$C$9*前提!$B$47,0)</f>
+        <f>ROUND(月別予算!$C$9*前提!$B$48,0)</f>
         <v/>
       </c>
       <c r="C12" s="27">
-        <f>ROUND(月別予算!$C$10*前提!$C$47,0)</f>
+        <f>ROUND(月別予算!$C$10*前提!$C$48,0)</f>
         <v/>
       </c>
       <c r="D12" s="27">
-        <f>ROUND(月別予算!$C$11*前提!$C$47,0)</f>
+        <f>ROUND(月別予算!$C$11*前提!$C$48,0)</f>
         <v/>
       </c>
       <c r="E12" s="27">
-        <f>ROUND(月別予算!$C$12*前提!$C$47,0)</f>
+        <f>ROUND(月別予算!$C$12*前提!$C$48,0)</f>
         <v/>
       </c>
       <c r="F12" s="27">
-        <f>ROUND(月別予算!$C$13*前提!$C$47,0)</f>
+        <f>ROUND(月別予算!$C$13*前提!$C$48,0)</f>
         <v/>
       </c>
       <c r="G12" s="27">
-        <f>ROUND(月別予算!$C$14*前提!$C$47,0)</f>
+        <f>ROUND(月別予算!$C$14*前提!$C$48,0)</f>
         <v/>
       </c>
       <c r="H12" s="27">
-        <f>ROUND(月別予算!$C$15*前提!$C$47,0)</f>
+        <f>ROUND(月別予算!$C$15*前提!$C$48,0)</f>
         <v/>
       </c>
       <c r="I12" s="27">
-        <f>ROUND(月別予算!$C$16*前提!$C$47,0)</f>
+        <f>ROUND(月別予算!$C$16*前提!$C$48,0)</f>
         <v/>
       </c>
       <c r="J12" s="28">

</xml_diff>

<commit_message>
Close September: final actuals in budget plan, October targets, full-month report
September normal operations finished at 637,248 yen (98% of budget). The
budget plan now uses the September actual (October becomes 801,761 yen),
targets.json switches to October, and the monthly report compares complete
months and reads each month's budget from its narrative file.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EFkMa7pBd48FUqtUrcDcW8
</commit_message>
<xml_diff>
--- a/reports/広告予算計画_2026-09改訂.xlsx
+++ b/reports/広告予算計画_2026-09改訂.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="前提" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="月別予算" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="FULLMARKS内訳" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="実施_日予算" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="9月実績" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="前提" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="月別予算" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FULLMARKS内訳" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="実施_日予算" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9月実績" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -590,11 +590,11 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>650000</v>
+        <v>637248</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>9/1〜9/24実績 ¥524,909（日割 ¥21,871）。残り6日 約2万円/日で月末 約64万の見込み。イベント枠は含まない</t>
+          <t>9月 確定実績 ¥637,248（日割 ¥21,241）。予算65万の98%。イベント枠は含まない</t>
         </is>
       </c>
     </row>
@@ -1522,7 +1522,7 @@
       </c>
       <c r="B9" s="18" t="inlineStr">
         <is>
-          <t>計画</t>
+          <t>実績</t>
         </is>
       </c>
       <c r="C9" s="19">
@@ -1563,7 +1563,7 @@
       </c>
       <c r="M9" s="17" t="inlineStr">
         <is>
-          <t>FULLMARKSのみ。9/1〜24実績 ¥524,909。SW企画は使用分 ¥48,422 を別枠で計上（予備費の残りは10〜4月へ）</t>
+          <t>FULLMARKSのみ。9月 確定実績 ¥637,248。SW企画は使用分 ¥48,422 を別枠で計上（予備費の残りは10〜4月へ）</t>
         </is>
       </c>
     </row>
@@ -4117,7 +4117,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>9月 実績（9/1〜9/24）と月換算</t>
+          <t>9月 確定実績（キャンペーン別）</t>
         </is>
       </c>
     </row>
@@ -4134,7 +4134,7 @@
       </c>
       <c r="C3" s="24" t="inlineStr">
         <is>
-          <t>9/1〜9/24 費用</t>
+          <t>9/1〜9/30 費用</t>
         </is>
       </c>
       <c r="D3" s="24" t="inlineStr">
@@ -4156,14 +4156,14 @@
       </c>
       <c r="B4" s="18" t="inlineStr">
         <is>
-          <t>UC_PL_5_PLA_v2</t>
+          <t>UC_SK_1_指名_フーディ二</t>
         </is>
       </c>
       <c r="C4" s="31" t="n">
-        <v>85598</v>
+        <v>102708</v>
       </c>
       <c r="D4" s="20">
-        <f>C4/24</f>
+        <f>C4/30</f>
         <v/>
       </c>
       <c r="E4" s="20">
@@ -4179,14 +4179,14 @@
       </c>
       <c r="B5" s="18" t="inlineStr">
         <is>
-          <t>UC_SK_1_指名_フーディ二</t>
+          <t>UC_PL_5_PLA_v2</t>
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>70344</v>
+        <v>89687</v>
       </c>
       <c r="D5" s="20">
-        <f>C5/24</f>
+        <f>C5/30</f>
         <v/>
       </c>
       <c r="E5" s="20">
@@ -4206,10 +4206,10 @@
         </is>
       </c>
       <c r="C6" s="31" t="n">
-        <v>60858</v>
+        <v>78045</v>
       </c>
       <c r="D6" s="20">
-        <f>C6/24</f>
+        <f>C6/30</f>
         <v/>
       </c>
       <c r="E6" s="20">
@@ -4229,10 +4229,10 @@
         </is>
       </c>
       <c r="C7" s="31" t="n">
-        <v>41556</v>
+        <v>47834</v>
       </c>
       <c r="D7" s="20">
-        <f>C7/24</f>
+        <f>C7/30</f>
         <v/>
       </c>
       <c r="E7" s="20">
@@ -4252,10 +4252,10 @@
         </is>
       </c>
       <c r="C8" s="31" t="n">
-        <v>8057</v>
+        <v>10780</v>
       </c>
       <c r="D8" s="20">
-        <f>C8/24</f>
+        <f>C8/30</f>
         <v/>
       </c>
       <c r="E8" s="20">
@@ -4275,10 +4275,10 @@
         </is>
       </c>
       <c r="C9" s="31" t="n">
-        <v>104104</v>
+        <v>129553</v>
       </c>
       <c r="D9" s="20">
-        <f>C9/24</f>
+        <f>C9/30</f>
         <v/>
       </c>
       <c r="E9" s="20">
@@ -4298,10 +4298,10 @@
         </is>
       </c>
       <c r="C10" s="31" t="n">
-        <v>49462</v>
+        <v>58865</v>
       </c>
       <c r="D10" s="20">
-        <f>C10/24</f>
+        <f>C10/30</f>
         <v/>
       </c>
       <c r="E10" s="20">
@@ -4317,14 +4317,14 @@
       </c>
       <c r="B11" s="18" t="inlineStr">
         <is>
-          <t>UC_DN_3_RTG_アクリマ_2608</t>
+          <t>UC_DN_4_CLK_アクリマ</t>
         </is>
       </c>
       <c r="C11" s="31" t="n">
-        <v>27751</v>
+        <v>33210</v>
       </c>
       <c r="D11" s="20">
-        <f>C11/24</f>
+        <f>C11/30</f>
         <v/>
       </c>
       <c r="E11" s="20">
@@ -4340,14 +4340,14 @@
       </c>
       <c r="B12" s="18" t="inlineStr">
         <is>
-          <t>UC_DN_4_CLK_アクリマ</t>
+          <t>UC_DN_3_RTG_ポック_2608</t>
         </is>
       </c>
       <c r="C12" s="31" t="n">
-        <v>27064</v>
+        <v>29286</v>
       </c>
       <c r="D12" s="20">
-        <f>C12/24</f>
+        <f>C12/30</f>
         <v/>
       </c>
       <c r="E12" s="20">
@@ -4363,14 +4363,14 @@
       </c>
       <c r="B13" s="18" t="inlineStr">
         <is>
-          <t>UC_DN_3_RTG_ポック_2608</t>
+          <t>UC_DN_3_RTG_ノローナ_2608</t>
         </is>
       </c>
       <c r="C13" s="31" t="n">
-        <v>25087</v>
+        <v>29093</v>
       </c>
       <c r="D13" s="20">
-        <f>C13/24</f>
+        <f>C13/30</f>
         <v/>
       </c>
       <c r="E13" s="20">
@@ -4386,14 +4386,14 @@
       </c>
       <c r="B14" s="18" t="inlineStr">
         <is>
-          <t>UC_DN_3_RTG_ノローナ_2608</t>
+          <t>UC_DN_3_RTG_アクリマ_2608</t>
         </is>
       </c>
       <c r="C14" s="31" t="n">
-        <v>24592</v>
+        <v>27751</v>
       </c>
       <c r="D14" s="20">
-        <f>C14/24</f>
+        <f>C14/30</f>
         <v/>
       </c>
       <c r="E14" s="20">
@@ -4416,7 +4416,7 @@
         <v>436</v>
       </c>
       <c r="D15" s="20">
-        <f>C15/24</f>
+        <f>C15/30</f>
         <v/>
       </c>
       <c r="E15" s="20">

</xml_diff>

<commit_message>
Roll October underspend into November-December in the budget plan
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EFkMa7pBd48FUqtUrcDcW8
</commit_message>
<xml_diff>
--- a/reports/広告予算計画_2026-09改訂.xlsx
+++ b/reports/広告予算計画_2026-09改訂.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -986,209 +986,228 @@
         <v/>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>10月 通常運用の確定実績（月末に入力。空欄なら計画どおり）</t>
+        </is>
+      </c>
+      <c r="B38" s="12" t="n"/>
+    </row>
     <row r="39">
-      <c r="A39" s="7" t="inlineStr">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>10月の使い残し（11月・12月に比率で上乗せ。2026-10-14 ユーザー指示）</t>
+        </is>
+      </c>
+      <c r="B39" s="10">
+        <f>IF(ISBLANK(前提!$B$38),0,前提!$B$37*前提!$B$29-前提!$B$38)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="inlineStr">
         <is>
           <t>FULLMARKS 内のブランド配分比率</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="9" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="9" t="inlineStr">
         <is>
           <t>ブランド/枠</t>
         </is>
       </c>
-      <c r="B40" s="9" t="inlineStr">
+      <c r="B42" s="9" t="inlineStr">
         <is>
           <t>9月 比率</t>
         </is>
       </c>
-      <c r="C40" s="9" t="inlineStr">
+      <c r="C42" s="9" t="inlineStr">
         <is>
           <t>10月〜 比率</t>
         </is>
       </c>
-      <c r="D40" s="9" t="inlineStr">
+      <c r="D42" s="9" t="inlineStr">
         <is>
           <t>備考</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="3" t="inlineStr">
-        <is>
-          <t>HOUDINI</t>
-        </is>
-      </c>
-      <c r="B41" s="5" t="n">
-        <v>0.27</v>
-      </c>
-      <c r="C41" s="5" t="n">
-        <v>0.26</v>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>広告売上の半分以上（9月 ROAS 11.8）。FULLMARKS で継続</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="3" t="inlineStr">
-        <is>
-          <t>商品連動(ショッピング/カタログ)</t>
-        </is>
-      </c>
-      <c r="B42" s="5" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="C42" s="5" t="n">
-        <v>0.23</v>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>通常価格品のみ（アウトレットは広告しない）。9月 ROAS: カタログ 4.6 / ショッピング 2.5。ショッピングを絞る</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>店舗指名(フルマークス)</t>
+          <t>HOUDINI</t>
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>0.17</v>
+        <v>0.27</v>
       </c>
       <c r="C43" s="5" t="n">
-        <v>0.18</v>
+        <v>0.26</v>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>9月 ROAS 16.2 の安定枠</t>
+          <t>広告売上の半分以上（9月 ROAS 11.8）。FULLMARKS で継続</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>POC</t>
+          <t>商品連動(ショッピング/カタログ)</t>
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>0.09</v>
+        <v>0.3</v>
       </c>
       <c r="C44" s="5" t="n">
-        <v>0.11</v>
+        <v>0.23</v>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>9月 ROAS 3.8。10月以降やや厚く</t>
+          <t>通常価格品のみ（アウトレットは広告しない）。9月 ROAS: カタログ 4.6 / ショッピング 2.5。ショッピングを絞る</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>NORRØNA</t>
+          <t>店舗指名(フルマークス)</t>
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.17</v>
       </c>
       <c r="C45" s="5" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.18</v>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>9月 ROAS 4.1（8月 1.0 から改善）。FULLMARKS で継続</t>
+          <t>9月 ROAS 16.2 の安定枠</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>ACLIMA</t>
+          <t>POC</t>
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>0.05</v>
+        <v>0.09</v>
       </c>
       <c r="C46" s="5" t="n">
-        <v>0.03</v>
+        <v>0.11</v>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>8〜9月の売上の72%がセール品、広告 ROAS 2.6。縮小</t>
+          <t>9月 ROAS 3.8。10月以降やや厚く</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>HESTRA【新規】</t>
+          <t>NORRØNA</t>
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>0.04</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="C47" s="5" t="n">
-        <v>0.1</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>10〜1月が本番。売上の79%が通常品（粗利50%）。フィード未掲載の解消が前提</t>
+          <t>9月 ROAS 4.1（8月 1.0 から改善）。FULLMARKS で継続</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>KANG【新規】</t>
+          <t>ACLIMA</t>
         </is>
       </c>
       <c r="B48" s="5" t="n">
-        <v>0.005</v>
+        <v>0.05</v>
       </c>
       <c r="C48" s="5" t="n">
-        <v>0.01</v>
+        <v>0.03</v>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>テスト枠</t>
+          <t>8〜9月の売上の72%がセール品、広告 ROAS 2.6。縮小</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
+          <t>HESTRA【新規】</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="C49" s="5" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>10〜1月が本番。売上の79%が通常品（粗利50%）。フィード未掲載の解消が前提</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>KANG【新規】</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="C50" s="5" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>テスト枠</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
           <t>PLUS ONE WORKS【新規】</t>
         </is>
       </c>
-      <c r="B49" s="5" t="n">
+      <c r="B51" s="5" t="n">
         <v>0.005</v>
       </c>
-      <c r="C49" s="5" t="n">
+      <c r="C51" s="5" t="n">
         <v>0.01</v>
       </c>
-      <c r="D49" s="2" t="inlineStr">
+      <c r="D51" s="2" t="inlineStr">
         <is>
           <t>テスト枠</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="7" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="7" t="inlineStr">
         <is>
           <t>計（各100%）</t>
         </is>
       </c>
-      <c r="B50" s="13">
-        <f>SUM(B41:B49)</f>
-        <v/>
-      </c>
-      <c r="C50" s="13">
-        <f>SUM(C41:C49)</f>
+      <c r="B52" s="13">
+        <f>SUM(B43:B51)</f>
+        <v/>
+      </c>
+      <c r="C52" s="13">
+        <f>SUM(C43:C51)</f>
         <v/>
       </c>
     </row>
@@ -1598,7 +1617,7 @@
         <v>0</v>
       </c>
       <c r="H10" s="20">
-        <f>前提!$B$37*前提!$B$29</f>
+        <f>IF(ISBLANK(前提!$B$38),前提!$B$37*前提!$B$29,前提!$B$38)</f>
         <v/>
       </c>
       <c r="I10" s="20" t="n">
@@ -1618,7 +1637,7 @@
       </c>
       <c r="M10" s="17" t="inlineStr">
         <is>
-          <t>冬物の立ち上がり前。約80万に抑え、11〜12月の通常品の冬物へ回す</t>
+          <t>冬物の立ち上がり前。約80万に抑え、使い残しも11〜12月の通常品の冬物へ回す（10/14 ユーザー指示）</t>
         </is>
       </c>
     </row>
@@ -1653,7 +1672,7 @@
         <v>0</v>
       </c>
       <c r="H11" s="20">
-        <f>前提!$B$37*前提!$B$30</f>
+        <f>前提!$B$37*前提!$B$30+前提!$B$39*前提!$B$30/(前提!$B$30+前提!$B$31)</f>
         <v/>
       </c>
       <c r="I11" s="19">
@@ -1672,7 +1691,11 @@
         <f>前提!$B$8-K11</f>
         <v/>
       </c>
-      <c r="M11" s="17" t="inlineStr"/>
+      <c r="M11" s="17" t="inlineStr">
+        <is>
+          <t>10月の使い残しを上乗せ（ブラックフライデー期間に厚く）</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="18" t="inlineStr">
@@ -1705,7 +1728,7 @@
         <v>0</v>
       </c>
       <c r="H12" s="20">
-        <f>前提!$B$37*前提!$B$31</f>
+        <f>前提!$B$37*前提!$B$31+前提!$B$39*前提!$B$31/(前提!$B$30+前提!$B$31)</f>
         <v/>
       </c>
       <c r="I12" s="19">
@@ -1726,7 +1749,7 @@
       </c>
       <c r="M12" s="17" t="inlineStr">
         <is>
-          <t>年末年始企画 予備10万</t>
+          <t>10月の使い残しを上乗せ。年末年始企画 予備10万</t>
         </is>
       </c>
     </row>
@@ -2103,35 +2126,35 @@
         </is>
       </c>
       <c r="B5" s="19">
-        <f>ROUND(月別予算!$C$9*前提!$B$41,0)</f>
+        <f>ROUND(月別予算!$C$9*前提!$B$43,0)</f>
         <v/>
       </c>
       <c r="C5" s="19">
-        <f>ROUND(月別予算!$C$10*前提!$C$41,0)</f>
+        <f>ROUND(月別予算!$C$10*前提!$C$43,0)</f>
         <v/>
       </c>
       <c r="D5" s="19">
-        <f>ROUND(月別予算!$C$11*前提!$C$41,0)</f>
+        <f>ROUND(月別予算!$C$11*前提!$C$43,0)</f>
         <v/>
       </c>
       <c r="E5" s="19">
-        <f>ROUND(月別予算!$C$12*前提!$C$41,0)</f>
+        <f>ROUND(月別予算!$C$12*前提!$C$43,0)</f>
         <v/>
       </c>
       <c r="F5" s="19">
-        <f>ROUND(月別予算!$C$13*前提!$C$41,0)</f>
+        <f>ROUND(月別予算!$C$13*前提!$C$43,0)</f>
         <v/>
       </c>
       <c r="G5" s="19">
-        <f>ROUND(月別予算!$C$14*前提!$C$41,0)</f>
+        <f>ROUND(月別予算!$C$14*前提!$C$43,0)</f>
         <v/>
       </c>
       <c r="H5" s="19">
-        <f>ROUND(月別予算!$C$15*前提!$C$41,0)</f>
+        <f>ROUND(月別予算!$C$15*前提!$C$43,0)</f>
         <v/>
       </c>
       <c r="I5" s="19">
-        <f>ROUND(月別予算!$C$16*前提!$C$41,0)</f>
+        <f>ROUND(月別予算!$C$16*前提!$C$43,0)</f>
         <v/>
       </c>
       <c r="J5" s="23">
@@ -2151,35 +2174,35 @@
         </is>
       </c>
       <c r="B6" s="19">
-        <f>ROUND(月別予算!$C$9*前提!$B$42,0)</f>
+        <f>ROUND(月別予算!$C$9*前提!$B$44,0)</f>
         <v/>
       </c>
       <c r="C6" s="19">
-        <f>ROUND(月別予算!$C$10*前提!$C$42,0)</f>
+        <f>ROUND(月別予算!$C$10*前提!$C$44,0)</f>
         <v/>
       </c>
       <c r="D6" s="19">
-        <f>ROUND(月別予算!$C$11*前提!$C$42,0)</f>
+        <f>ROUND(月別予算!$C$11*前提!$C$44,0)</f>
         <v/>
       </c>
       <c r="E6" s="19">
-        <f>ROUND(月別予算!$C$12*前提!$C$42,0)</f>
+        <f>ROUND(月別予算!$C$12*前提!$C$44,0)</f>
         <v/>
       </c>
       <c r="F6" s="19">
-        <f>ROUND(月別予算!$C$13*前提!$C$42,0)</f>
+        <f>ROUND(月別予算!$C$13*前提!$C$44,0)</f>
         <v/>
       </c>
       <c r="G6" s="19">
-        <f>ROUND(月別予算!$C$14*前提!$C$42,0)</f>
+        <f>ROUND(月別予算!$C$14*前提!$C$44,0)</f>
         <v/>
       </c>
       <c r="H6" s="19">
-        <f>ROUND(月別予算!$C$15*前提!$C$42,0)</f>
+        <f>ROUND(月別予算!$C$15*前提!$C$44,0)</f>
         <v/>
       </c>
       <c r="I6" s="19">
-        <f>ROUND(月別予算!$C$16*前提!$C$42,0)</f>
+        <f>ROUND(月別予算!$C$16*前提!$C$44,0)</f>
         <v/>
       </c>
       <c r="J6" s="23">
@@ -2199,35 +2222,35 @@
         </is>
       </c>
       <c r="B7" s="19">
-        <f>ROUND(月別予算!$C$9*前提!$B$43,0)</f>
+        <f>ROUND(月別予算!$C$9*前提!$B$45,0)</f>
         <v/>
       </c>
       <c r="C7" s="19">
-        <f>ROUND(月別予算!$C$10*前提!$C$43,0)</f>
+        <f>ROUND(月別予算!$C$10*前提!$C$45,0)</f>
         <v/>
       </c>
       <c r="D7" s="19">
-        <f>ROUND(月別予算!$C$11*前提!$C$43,0)</f>
+        <f>ROUND(月別予算!$C$11*前提!$C$45,0)</f>
         <v/>
       </c>
       <c r="E7" s="19">
-        <f>ROUND(月別予算!$C$12*前提!$C$43,0)</f>
+        <f>ROUND(月別予算!$C$12*前提!$C$45,0)</f>
         <v/>
       </c>
       <c r="F7" s="19">
-        <f>ROUND(月別予算!$C$13*前提!$C$43,0)</f>
+        <f>ROUND(月別予算!$C$13*前提!$C$45,0)</f>
         <v/>
       </c>
       <c r="G7" s="19">
-        <f>ROUND(月別予算!$C$14*前提!$C$43,0)</f>
+        <f>ROUND(月別予算!$C$14*前提!$C$45,0)</f>
         <v/>
       </c>
       <c r="H7" s="19">
-        <f>ROUND(月別予算!$C$15*前提!$C$43,0)</f>
+        <f>ROUND(月別予算!$C$15*前提!$C$45,0)</f>
         <v/>
       </c>
       <c r="I7" s="19">
-        <f>ROUND(月別予算!$C$16*前提!$C$43,0)</f>
+        <f>ROUND(月別予算!$C$16*前提!$C$45,0)</f>
         <v/>
       </c>
       <c r="J7" s="23">
@@ -2247,35 +2270,35 @@
         </is>
       </c>
       <c r="B8" s="19">
-        <f>ROUND(月別予算!$C$9*前提!$B$44,0)</f>
+        <f>ROUND(月別予算!$C$9*前提!$B$46,0)</f>
         <v/>
       </c>
       <c r="C8" s="19">
-        <f>ROUND(月別予算!$C$10*前提!$C$44,0)</f>
+        <f>ROUND(月別予算!$C$10*前提!$C$46,0)</f>
         <v/>
       </c>
       <c r="D8" s="19">
-        <f>ROUND(月別予算!$C$11*前提!$C$44,0)</f>
+        <f>ROUND(月別予算!$C$11*前提!$C$46,0)</f>
         <v/>
       </c>
       <c r="E8" s="19">
-        <f>ROUND(月別予算!$C$12*前提!$C$44,0)</f>
+        <f>ROUND(月別予算!$C$12*前提!$C$46,0)</f>
         <v/>
       </c>
       <c r="F8" s="19">
-        <f>ROUND(月別予算!$C$13*前提!$C$44,0)</f>
+        <f>ROUND(月別予算!$C$13*前提!$C$46,0)</f>
         <v/>
       </c>
       <c r="G8" s="19">
-        <f>ROUND(月別予算!$C$14*前提!$C$44,0)</f>
+        <f>ROUND(月別予算!$C$14*前提!$C$46,0)</f>
         <v/>
       </c>
       <c r="H8" s="19">
-        <f>ROUND(月別予算!$C$15*前提!$C$44,0)</f>
+        <f>ROUND(月別予算!$C$15*前提!$C$46,0)</f>
         <v/>
       </c>
       <c r="I8" s="19">
-        <f>ROUND(月別予算!$C$16*前提!$C$44,0)</f>
+        <f>ROUND(月別予算!$C$16*前提!$C$46,0)</f>
         <v/>
       </c>
       <c r="J8" s="23">
@@ -2295,35 +2318,35 @@
         </is>
       </c>
       <c r="B9" s="19">
-        <f>ROUND(月別予算!$C$9*前提!$B$45,0)</f>
+        <f>ROUND(月別予算!$C$9*前提!$B$47,0)</f>
         <v/>
       </c>
       <c r="C9" s="19">
-        <f>ROUND(月別予算!$C$10*前提!$C$45,0)</f>
+        <f>ROUND(月別予算!$C$10*前提!$C$47,0)</f>
         <v/>
       </c>
       <c r="D9" s="19">
-        <f>ROUND(月別予算!$C$11*前提!$C$45,0)</f>
+        <f>ROUND(月別予算!$C$11*前提!$C$47,0)</f>
         <v/>
       </c>
       <c r="E9" s="19">
-        <f>ROUND(月別予算!$C$12*前提!$C$45,0)</f>
+        <f>ROUND(月別予算!$C$12*前提!$C$47,0)</f>
         <v/>
       </c>
       <c r="F9" s="19">
-        <f>ROUND(月別予算!$C$13*前提!$C$45,0)</f>
+        <f>ROUND(月別予算!$C$13*前提!$C$47,0)</f>
         <v/>
       </c>
       <c r="G9" s="19">
-        <f>ROUND(月別予算!$C$14*前提!$C$45,0)</f>
+        <f>ROUND(月別予算!$C$14*前提!$C$47,0)</f>
         <v/>
       </c>
       <c r="H9" s="19">
-        <f>ROUND(月別予算!$C$15*前提!$C$45,0)</f>
+        <f>ROUND(月別予算!$C$15*前提!$C$47,0)</f>
         <v/>
       </c>
       <c r="I9" s="19">
-        <f>ROUND(月別予算!$C$16*前提!$C$45,0)</f>
+        <f>ROUND(月別予算!$C$16*前提!$C$47,0)</f>
         <v/>
       </c>
       <c r="J9" s="23">
@@ -2343,35 +2366,35 @@
         </is>
       </c>
       <c r="B10" s="19">
-        <f>ROUND(月別予算!$C$9*前提!$B$46,0)</f>
+        <f>ROUND(月別予算!$C$9*前提!$B$48,0)</f>
         <v/>
       </c>
       <c r="C10" s="19">
-        <f>ROUND(月別予算!$C$10*前提!$C$46,0)</f>
+        <f>ROUND(月別予算!$C$10*前提!$C$48,0)</f>
         <v/>
       </c>
       <c r="D10" s="19">
-        <f>ROUND(月別予算!$C$11*前提!$C$46,0)</f>
+        <f>ROUND(月別予算!$C$11*前提!$C$48,0)</f>
         <v/>
       </c>
       <c r="E10" s="19">
-        <f>ROUND(月別予算!$C$12*前提!$C$46,0)</f>
+        <f>ROUND(月別予算!$C$12*前提!$C$48,0)</f>
         <v/>
       </c>
       <c r="F10" s="19">
-        <f>ROUND(月別予算!$C$13*前提!$C$46,0)</f>
+        <f>ROUND(月別予算!$C$13*前提!$C$48,0)</f>
         <v/>
       </c>
       <c r="G10" s="19">
-        <f>ROUND(月別予算!$C$14*前提!$C$46,0)</f>
+        <f>ROUND(月別予算!$C$14*前提!$C$48,0)</f>
         <v/>
       </c>
       <c r="H10" s="19">
-        <f>ROUND(月別予算!$C$15*前提!$C$46,0)</f>
+        <f>ROUND(月別予算!$C$15*前提!$C$48,0)</f>
         <v/>
       </c>
       <c r="I10" s="19">
-        <f>ROUND(月別予算!$C$16*前提!$C$46,0)</f>
+        <f>ROUND(月別予算!$C$16*前提!$C$48,0)</f>
         <v/>
       </c>
       <c r="J10" s="23">
@@ -2391,35 +2414,35 @@
         </is>
       </c>
       <c r="B11" s="27">
-        <f>ROUND(月別予算!$C$9*前提!$B$47,0)</f>
+        <f>ROUND(月別予算!$C$9*前提!$B$49,0)</f>
         <v/>
       </c>
       <c r="C11" s="27">
-        <f>ROUND(月別予算!$C$10*前提!$C$47,0)</f>
+        <f>ROUND(月別予算!$C$10*前提!$C$49,0)</f>
         <v/>
       </c>
       <c r="D11" s="27">
-        <f>ROUND(月別予算!$C$11*前提!$C$47,0)</f>
+        <f>ROUND(月別予算!$C$11*前提!$C$49,0)</f>
         <v/>
       </c>
       <c r="E11" s="27">
-        <f>ROUND(月別予算!$C$12*前提!$C$47,0)</f>
+        <f>ROUND(月別予算!$C$12*前提!$C$49,0)</f>
         <v/>
       </c>
       <c r="F11" s="27">
-        <f>ROUND(月別予算!$C$13*前提!$C$47,0)</f>
+        <f>ROUND(月別予算!$C$13*前提!$C$49,0)</f>
         <v/>
       </c>
       <c r="G11" s="27">
-        <f>ROUND(月別予算!$C$14*前提!$C$47,0)</f>
+        <f>ROUND(月別予算!$C$14*前提!$C$49,0)</f>
         <v/>
       </c>
       <c r="H11" s="27">
-        <f>ROUND(月別予算!$C$15*前提!$C$47,0)</f>
+        <f>ROUND(月別予算!$C$15*前提!$C$49,0)</f>
         <v/>
       </c>
       <c r="I11" s="27">
-        <f>ROUND(月別予算!$C$16*前提!$C$47,0)</f>
+        <f>ROUND(月別予算!$C$16*前提!$C$49,0)</f>
         <v/>
       </c>
       <c r="J11" s="28">
@@ -2439,35 +2462,35 @@
         </is>
       </c>
       <c r="B12" s="27">
-        <f>ROUND(月別予算!$C$9*前提!$B$48,0)</f>
+        <f>ROUND(月別予算!$C$9*前提!$B$50,0)</f>
         <v/>
       </c>
       <c r="C12" s="27">
-        <f>ROUND(月別予算!$C$10*前提!$C$48,0)</f>
+        <f>ROUND(月別予算!$C$10*前提!$C$50,0)</f>
         <v/>
       </c>
       <c r="D12" s="27">
-        <f>ROUND(月別予算!$C$11*前提!$C$48,0)</f>
+        <f>ROUND(月別予算!$C$11*前提!$C$50,0)</f>
         <v/>
       </c>
       <c r="E12" s="27">
-        <f>ROUND(月別予算!$C$12*前提!$C$48,0)</f>
+        <f>ROUND(月別予算!$C$12*前提!$C$50,0)</f>
         <v/>
       </c>
       <c r="F12" s="27">
-        <f>ROUND(月別予算!$C$13*前提!$C$48,0)</f>
+        <f>ROUND(月別予算!$C$13*前提!$C$50,0)</f>
         <v/>
       </c>
       <c r="G12" s="27">
-        <f>ROUND(月別予算!$C$14*前提!$C$48,0)</f>
+        <f>ROUND(月別予算!$C$14*前提!$C$50,0)</f>
         <v/>
       </c>
       <c r="H12" s="27">
-        <f>ROUND(月別予算!$C$15*前提!$C$48,0)</f>
+        <f>ROUND(月別予算!$C$15*前提!$C$50,0)</f>
         <v/>
       </c>
       <c r="I12" s="27">
-        <f>ROUND(月別予算!$C$16*前提!$C$48,0)</f>
+        <f>ROUND(月別予算!$C$16*前提!$C$50,0)</f>
         <v/>
       </c>
       <c r="J12" s="28">

</xml_diff>